<commit_message>
Set confirmed week end date 06/07/2026 and add hours-discrepancy note to LCPtracker file
https://claude.ai/code/session_019s5PB6c6irLf4S2x8maUct
</commit_message>
<xml_diff>
--- a/output/LCPtracker_ORBA_ELECTRIC_20260609.xlsx
+++ b/output/LCPtracker_ORBA_ELECTRIC_20260609.xlsx
@@ -961,11 +961,9 @@
           <t>[MISSING - get from LCPtracker admin]</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>[MISSING - confirm week end date e.g. 06/07/2026]</t>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>06/07/2026</t>
         </is>
       </c>
       <c r="F2" s="3" t="n">
@@ -1163,7 +1161,6 @@
           <t>[MISSING - client has]</t>
         </is>
       </c>
-      <c r="BI2" t="inlineStr"/>
       <c r="BJ2" s="2" t="inlineStr">
         <is>
           <t>[MISSING - client has]</t>
@@ -1194,7 +1191,6 @@
           <t>[MISSING - client has]</t>
         </is>
       </c>
-      <c r="BP2" t="inlineStr"/>
       <c r="BQ2" s="2" t="inlineStr">
         <is>
           <t>[MISSING - confirm with LCPtracker admin]</t>
@@ -1224,8 +1220,6 @@
       <c r="BY2" s="3" t="n">
         <v>70.28</v>
       </c>
-      <c r="BZ2" t="inlineStr"/>
-      <c r="CA2" t="inlineStr"/>
       <c r="CB2" s="2" t="inlineStr">
         <is>
           <t>[MISSING - client has]</t>
@@ -1241,9 +1235,6 @@
           <t>New York</t>
         </is>
       </c>
-      <c r="CE2" t="inlineStr"/>
-      <c r="CF2" t="inlineStr"/>
-      <c r="CG2" t="inlineStr"/>
       <c r="CH2" s="3" t="inlineStr">
         <is>
           <t>NYC Resident LIT=$102.00; NY PFL=$11.40; NY Vol Disability=$0.60</t>
@@ -1254,28 +1245,16 @@
           <t>[MISSING - from W-4]</t>
         </is>
       </c>
-      <c r="CJ2" t="inlineStr"/>
-      <c r="CK2" t="inlineStr"/>
       <c r="CL2" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="CM2" t="inlineStr"/>
-      <c r="CN2" t="inlineStr"/>
-      <c r="CO2" t="inlineStr"/>
-      <c r="CP2" t="inlineStr"/>
-      <c r="CQ2" t="inlineStr"/>
-      <c r="CR2" t="inlineStr"/>
-      <c r="CS2" t="inlineStr"/>
-      <c r="CT2" t="inlineStr"/>
-      <c r="CU2" t="inlineStr"/>
       <c r="CV2" s="2" t="inlineStr">
         <is>
           <t>[MISSING - confirm if IBEW Local 3]</t>
         </is>
       </c>
-      <c r="CW2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
@@ -1283,11 +1262,9 @@
           <t>[MISSING - get from LCPtracker admin]</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>[MISSING - confirm week end date e.g. 06/07/2026]</t>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>06/07/2026</t>
         </is>
       </c>
       <c r="F3" s="3" t="n">
@@ -1485,7 +1462,6 @@
           <t>[MISSING - client has]</t>
         </is>
       </c>
-      <c r="BI3" t="inlineStr"/>
       <c r="BJ3" s="2" t="inlineStr">
         <is>
           <t>[MISSING - client has]</t>
@@ -1516,7 +1492,6 @@
           <t>[MISSING - client has]</t>
         </is>
       </c>
-      <c r="BP3" t="inlineStr"/>
       <c r="BQ3" s="2" t="inlineStr">
         <is>
           <t>[MISSING - confirm with LCPtracker admin]</t>
@@ -1546,8 +1521,6 @@
       <c r="BY3" s="3" t="n">
         <v>70.28</v>
       </c>
-      <c r="BZ3" t="inlineStr"/>
-      <c r="CA3" t="inlineStr"/>
       <c r="CB3" s="2" t="inlineStr">
         <is>
           <t>[MISSING - client has]</t>
@@ -1563,9 +1536,6 @@
           <t>New York</t>
         </is>
       </c>
-      <c r="CE3" t="inlineStr"/>
-      <c r="CF3" t="inlineStr"/>
-      <c r="CG3" t="inlineStr"/>
       <c r="CH3" s="3" t="inlineStr">
         <is>
           <t>NYC Resident LIT=$102.00; NY PFL=$11.40; NY Vol Disability=$0.60</t>
@@ -1576,28 +1546,16 @@
           <t>[MISSING - from W-4]</t>
         </is>
       </c>
-      <c r="CJ3" t="inlineStr"/>
-      <c r="CK3" t="inlineStr"/>
       <c r="CL3" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="CM3" t="inlineStr"/>
-      <c r="CN3" t="inlineStr"/>
-      <c r="CO3" t="inlineStr"/>
-      <c r="CP3" t="inlineStr"/>
-      <c r="CQ3" t="inlineStr"/>
-      <c r="CR3" t="inlineStr"/>
-      <c r="CS3" t="inlineStr"/>
-      <c r="CT3" t="inlineStr"/>
-      <c r="CU3" t="inlineStr"/>
       <c r="CV3" s="2" t="inlineStr">
         <is>
           <t>[MISSING - confirm if IBEW Local 3]</t>
         </is>
       </c>
-      <c r="CW3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -1627,7 +1585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B45"/>
+  <dimension ref="A1:B49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1641,9 +1599,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1867,9 +1823,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr"/>
-    </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
@@ -1897,7 +1851,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Confirm the week end date — likely 06/07/2026 (Sat) or 06/08/2026 (Sun)</t>
+          <t>CONFIRMED: 06/07/2026 (pay period 6/1-6/7) — already entered in Sheet1</t>
         </is>
       </c>
     </row>
@@ -2045,9 +1999,7 @@
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr"/>
-    </row>
+    <row r="38"/>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
@@ -2094,6 +2046,27 @@
       <c r="A45" t="inlineStr">
         <is>
           <t xml:space="preserve">  6. Both employees have identical pay — only check number and personal info differ</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>HOURS NOTE: ADP stub shows 55.5 total hours because 18.5 hrs was entered under all 3 earning codes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Actual hours worked = 18.5. LCPtracker upload uses 18.5 (correct). For future payrolls, put hours</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>only on Regular and enter Supplemental + 6.2% Fringe as flat dollar amounts so the stub matches.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update LCPtracker template with employee data from pay stubs
Added addresses (Cruz: Staten Island, Solomon: Brooklyn), contract ID C224300,
work county Kings, W-4 exemptions. Updated NOTES tab with remaining missing fields
and class_code troubleshooting guidance.

https://claude.ai/code/session_019s5PB6c6irLf4S2x8maUct
</commit_message>
<xml_diff>
--- a/output/LCPtracker_ORBA_ELECTRIC_20260609.xlsx
+++ b/output/LCPtracker_ORBA_ELECTRIC_20260609.xlsx
@@ -958,7 +958,12 @@
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>[MISSING - get from LCPtracker admin]</t>
+          <t>C224300 [VERIFY in LCPtracker]</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>C224300</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -1148,32 +1153,33 @@
       </c>
       <c r="BF2" s="3" t="inlineStr">
         <is>
-          <t>[CRUZ]</t>
+          <t>Cesar</t>
         </is>
       </c>
       <c r="BG2" s="3" t="inlineStr">
         <is>
-          <t>[CESAR]</t>
-        </is>
-      </c>
-      <c r="BH2" s="2" t="inlineStr">
-        <is>
-          <t>[MISSING - client has]</t>
-        </is>
-      </c>
-      <c r="BJ2" s="2" t="inlineStr">
-        <is>
-          <t>[MISSING - client has]</t>
-        </is>
-      </c>
-      <c r="BK2" s="2" t="inlineStr">
-        <is>
-          <t>[MISSING - client has]</t>
-        </is>
-      </c>
-      <c r="BL2" s="2" t="inlineStr">
-        <is>
-          <t>[MISSING - client has]</t>
+          <t>Cruz</t>
+        </is>
+      </c>
+      <c r="BH2" s="3" t="inlineStr">
+        <is>
+          <t>976 South Railroad Avenue</t>
+        </is>
+      </c>
+      <c r="BI2" s="3" t="inlineStr"/>
+      <c r="BJ2" s="3" t="inlineStr">
+        <is>
+          <t>Staten Island</t>
+        </is>
+      </c>
+      <c r="BK2" s="3" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="BL2" s="3" t="inlineStr">
+        <is>
+          <t>10306</t>
         </is>
       </c>
       <c r="BM2" s="2" t="inlineStr">
@@ -1232,7 +1238,7 @@
       </c>
       <c r="CD2" s="3" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Kings</t>
         </is>
       </c>
       <c r="CH2" s="3" t="inlineStr">
@@ -1240,9 +1246,9 @@
           <t>NYC Resident LIT=$102.00; NY PFL=$11.40; NY Vol Disability=$0.60</t>
         </is>
       </c>
-      <c r="CI2" s="2" t="inlineStr">
-        <is>
-          <t>[MISSING - from W-4]</t>
+      <c r="CI2" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
       <c r="CL2" s="3" t="inlineStr">
@@ -1259,7 +1265,12 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>[MISSING - get from LCPtracker admin]</t>
+          <t>C224300 [VERIFY in LCPtracker]</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>C224300</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -1449,32 +1460,33 @@
       </c>
       <c r="BF3" s="3" t="inlineStr">
         <is>
-          <t>[LEEOR]</t>
+          <t>Leeor</t>
         </is>
       </c>
       <c r="BG3" s="3" t="inlineStr">
         <is>
-          <t>[SOLOMON]</t>
-        </is>
-      </c>
-      <c r="BH3" s="2" t="inlineStr">
-        <is>
-          <t>[MISSING - client has]</t>
-        </is>
-      </c>
-      <c r="BJ3" s="2" t="inlineStr">
-        <is>
-          <t>[MISSING - client has]</t>
-        </is>
-      </c>
-      <c r="BK3" s="2" t="inlineStr">
-        <is>
-          <t>[MISSING - client has]</t>
-        </is>
-      </c>
-      <c r="BL3" s="2" t="inlineStr">
-        <is>
-          <t>[MISSING - client has]</t>
+          <t>SOLOMON</t>
+        </is>
+      </c>
+      <c r="BH3" s="3" t="inlineStr">
+        <is>
+          <t>2739 64th St</t>
+        </is>
+      </c>
+      <c r="BI3" s="3" t="inlineStr"/>
+      <c r="BJ3" s="3" t="inlineStr">
+        <is>
+          <t>Brooklyn</t>
+        </is>
+      </c>
+      <c r="BK3" s="3" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="BL3" s="3" t="inlineStr">
+        <is>
+          <t>11234</t>
         </is>
       </c>
       <c r="BM3" s="2" t="inlineStr">
@@ -1533,7 +1545,7 @@
       </c>
       <c r="CD3" s="3" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Kings</t>
         </is>
       </c>
       <c r="CH3" s="3" t="inlineStr">
@@ -1541,9 +1553,9 @@
           <t>NYC Resident LIT=$102.00; NY PFL=$11.40; NY Vol Disability=$0.60</t>
         </is>
       </c>
-      <c r="CI3" s="2" t="inlineStr">
-        <is>
-          <t>[MISSING - from W-4]</t>
+      <c r="CI3" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
       <c r="CL3" s="3" t="inlineStr">
@@ -1585,7 +1597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B49"/>
+  <dimension ref="A1:B74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1599,7 +1611,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1823,7 +1834,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
@@ -1999,7 +2009,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
@@ -2067,6 +2076,227 @@
       <c r="A49" t="inlineStr">
         <is>
           <t>only on Regular and enter Supplemental + 6.2% Fringe as flat dollar amounts so the stub matches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>UPDATED FROM PAY STUBS (6/11/2026):</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Cesar Cruz address</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>976 South Railroad Avenue, Staten Island, NY 10306</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Leeor Solomon address</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2739 64th St, Brooklyn, NY 11234</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  contract_id</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>C224300 (IN-SITU SOIL STABILIZATION, 37 Otsego St)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  project_code</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>C224300 used as placeholder — MUST verify in LCPtracker against actual project code</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  work_county</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Kings (Brooklyn — job site at 37 Otsego St)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  num_exempt</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>0 (Federal Std W/H Table, State 0, Local 0 per pay stubs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>STILL MISSING:</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SSN</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>You have them — type into column G (format: XXX-XX-XXXX)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  employee_ID</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Look up each employee in ADP RUN &gt; Employee Profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  class_code / craft_id</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>CRITICAL — must be mapped in LCPtracker before upload or it will fail. Contact LCPtracker admin or project GC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  st_hrs_date1-7</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Daily hour split totaling 18.5 hrs — Leeor has the timesheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  phone</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>From ADP employee profiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  gender / ethnicity</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>From ADP employee profiles (required for NYC compliance)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  date_hired</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>From ADP employee profiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>CLASS CODE NOTE:</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  This is the #1 reason LCPtracker uploads fail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  The code you enter must exactly match what the prime contractor or LCPtracker admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  has mapped under Setup &gt; Craft Matching for this project.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  For Electrician A rate on a NYC public works job, it is likely mapped as ELEC or similar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Call LCPtracker support at 714-669-0052 option 4 and give them contract #C224300.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Enter SSNs and ADP employee IDs into LCPtracker template
https://claude.ai/code/session_019s5PB6c6irLf4S2x8maUct
</commit_message>
<xml_diff>
--- a/output/LCPtracker_ORBA_ELECTRIC_20260609.xlsx
+++ b/output/LCPtracker_ORBA_ELECTRIC_20260609.xlsx
@@ -974,14 +974,14 @@
       <c r="F2" s="3" t="n">
         <v>50001</v>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>[MISSING - client has]</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>[MISSING - look up in ADP employee profile]</t>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>069-94-7686</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -1281,14 +1281,14 @@
       <c r="F3" s="3" t="n">
         <v>50002</v>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>[MISSING - client has]</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>[MISSING - look up in ADP employee profile]</t>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>087-70-0559</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -2079,9 +2079,7 @@
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="inlineStr"/>
-    </row>
+    <row r="51"/>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
@@ -2161,9 +2159,7 @@
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" t="inlineStr"/>
-    </row>
+    <row r="59"/>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
@@ -2255,9 +2251,7 @@
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" t="inlineStr"/>
-    </row>
+    <row r="68"/>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Swap employee IDs (Cruz=2, Solomon=1) and remove SSNs for email-safe version
https://claude.ai/code/session_019s5PB6c6irLf4S2x8maUct
</commit_message>
<xml_diff>
--- a/output/LCPtracker_ORBA_ELECTRIC_20260609.xlsx
+++ b/output/LCPtracker_ORBA_ELECTRIC_20260609.xlsx
@@ -974,14 +974,14 @@
       <c r="F2" s="3" t="n">
         <v>50001</v>
       </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>069-94-7686</t>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>[ENTER SSN]</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -1281,14 +1281,14 @@
       <c r="F3" s="3" t="n">
         <v>50002</v>
       </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>087-70-0559</t>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>[ENTER SSN]</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -2079,7 +2079,6 @@
         </is>
       </c>
     </row>
-    <row r="51"/>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
@@ -2159,7 +2158,6 @@
         </is>
       </c>
     </row>
-    <row r="59"/>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
@@ -2251,7 +2249,6 @@
         </is>
       </c>
     </row>
-    <row r="68"/>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>

</xml_diff>